<commit_message>
Generacion de resguardo funcional
siiiiii
</commit_message>
<xml_diff>
--- a/database/controller_excel/Plantilla3.xlsx
+++ b/database/controller_excel/Plantilla3.xlsx
@@ -10,6 +10,10 @@
   <sheets>
     <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="false" name="area" vbProcedure="false">Hoja1!$G$38</definedName>
+    <definedName function="false" hidden="false" name="nombre" vbProcedure="false">Hoja1!$G$37</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -20,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t xml:space="preserve">SERVICIOS PETROLEROS TERRESTES</t>
   </si>
@@ -119,9 +123,6 @@
   </si>
   <si>
     <t xml:space="preserve">Supervisor TI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propuestas Técnicas</t>
   </si>
 </sst>
 </file>
@@ -465,9 +466,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>865800</xdr:colOff>
+      <xdr:colOff>864360</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>84600</xdr:rowOff>
+      <xdr:rowOff>83160</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -481,7 +482,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="114480" y="285840"/>
-          <a:ext cx="751320" cy="751320"/>
+          <a:ext cx="749880" cy="749880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -678,12 +679,12 @@
   <sheetFormatPr defaultColWidth="10.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="21.57"/>
   </cols>
   <sheetData>
@@ -1173,8 +1174,9 @@
       <c r="D38" s="37"/>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
-      <c r="G38" s="37" t="s">
-        <v>33</v>
+      <c r="G38" s="37" t="str">
+        <f aca="false">C12</f>
+        <v>Propuestas Tecnicas</v>
       </c>
       <c r="H38" s="37"/>
       <c r="I38" s="37"/>

</xml_diff>